<commit_message>
docs: state the board control in C10 rather than a count that goes stale
Raised by Tristan in review of #23. The cell asserted "all eighteen issues are
on the board". The repository now holds twenty-one, and two of them (#27 and
#32) were not on the board at all, so the claim was not merely out of date but
untrue at the moment it was read.

The board itself is corrected: every issue is now on it, which needed no code
change.

The cell no longer states a number. A count is wrong the moment anyone opens an
issue, and evidence that expires on its own is weaker than evidence describing
the control that holds. It now records that every issue raised is placed on the
board and that each controlled change references its issue from the branch and
the Pull Request, which stays true as the project grows.

Refs: #23, #6, #27, #32
</commit_message>
<xml_diff>
--- a/docs/requirements/CivicConnect_M1_Registers.xlsx
+++ b/docs/requirements/CivicConnect_M1_Registers.xlsx
@@ -88,7 +88,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1753" uniqueCount="996">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1753" uniqueCount="997">
   <si>
     <t xml:space="preserve">CivicConnect - Milestone 1 controlled registers</t>
   </si>
@@ -3076,6 +3076,9 @@
   </si>
   <si>
     <t xml:space="preserve">https://github.com/PVY-Smit/civicconnect/tree/main/docs. docs/PED, docs/requirements, docs/architecture, docs/decisions, docs/risk, docs/change, docs/quality, docs/security, docs/deployment, plus src/, tests/ and .github/. Folders for later milestones are present and empty by design (Master Brief, Appendix C).</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Board: https://github.com/users/PVY-Smit/projects/1. Issues: https://github.com/PVY-Smit/civicconnect/issues. Every issue raised on the project is placed on the board, and each controlled change references its issue from the branch name and from the Pull Request that implements it. No fixed count is stated here: the number changes whenever an issue is raised, and evidence that goes stale on its own is weaker than evidence that describes the control.</t>
   </si>
 </sst>
 </file>
@@ -5582,7 +5585,7 @@
         <v>899</v>
       </c>
       <c r="C10" s="10" t="s">
-        <v>991</v>
+        <v>996</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">

</xml_diff>

<commit_message>
docs: complete the last GitHub Governance evidence cell
C12, the review checklist, was the one cell of twelve left deliberately open in
#23. There was no review comment to link to, so the control was configured but
had not operated, and pointing the cell at the checklist text would have
answered a question the criterion does not ask.

The control has now operated. Review of #18 found the registers-updated
checklist inverted against the actual change, which was corrected in response,
and found that the Figure 2 label defect was recorded inside a register row
without being tracked as work, which is now issue #27.

The cell cites both, plus an approval carrying reasoning rather than a bare
tick, because Master Brief s9 makes review quality part of the control: an
approval that does not reflect meaningful review may receive no credit.

All twelve cells are now complete and no cell in the sheet remains flagged as
outstanding.

Refs: #6, #18, #19, #27
</commit_message>
<xml_diff>
--- a/docs/requirements/CivicConnect_M1_Registers.xlsx
+++ b/docs/requirements/CivicConnect_M1_Registers.xlsx
@@ -88,7 +88,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1753" uniqueCount="997">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1753" uniqueCount="998">
   <si>
     <t xml:space="preserve">CivicConnect - Milestone 1 controlled registers</t>
   </si>
@@ -3079,6 +3079,9 @@
   </si>
   <si>
     <t xml:space="preserve">Board: https://github.com/users/PVY-Smit/projects/1. Issues: https://github.com/PVY-Smit/civicconnect/issues. Every issue raised on the project is placed on the board, and each controlled change references its issue from the branch name and from the Pull Request that implements it. No fixed count is stated here: the number changes whenever an issue is raised, and evidence that goes stale on its own is weaker than evidence that describes the control.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Checklist in CONTRIBUTING.md, "Review checklist": https://github.com/PVY-Smit/civicconnect/blob/800b982f60ff7edb1931debc8525ffb6a48a5a20/CONTRIBUTING.md#L55-L68. The control operating, not merely configured: review of #18 found the registers-updated checklist inverted against the actual change, which was corrected in response (https://github.com/PVY-Smit/civicconnect/pull/18#issuecomment-5583144236); the same review found that the Figure 2 label defect was recorded in a register row but not tracked as work, and it was raised as issue #27 (https://github.com/PVY-Smit/civicconnect/pull/18#issuecomment-5583171255). Approval carrying reasoning rather than a bare tick: https://github.com/PVY-Smit/civicconnect/pull/19#pullrequestreview-5140293911.</t>
   </si>
 </sst>
 </file>
@@ -5606,8 +5609,8 @@
       <c r="B12" s="10" t="s">
         <v>905</v>
       </c>
-      <c r="C12" s="12" t="s">
-        <v>993</v>
+      <c r="C12" s="10" t="s">
+        <v>997</v>
       </c>
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">

</xml_diff>

<commit_message>
docs: complete Tristan AI Usage Register entry
Records Tristan Roets's M1 AI-assisted work in the controlled register and the
PED s14.2 mirror: the engineering task, what the assistant contributed, the
independent verification applied, and what was accepted after revision or
rejected.

Content supplied by Tristan Roets. Committed from Jean Smit's account because
he could not reach a machine tonight, and at his explicit request the commit is
not attributed to him: the authorship reflects who made the commit, and this
message records whose work it is.

His verification is checked against the live repository rather than asserted,
and the issues-found column records that some assistant output rested on an
outdated view of repository state and was corrected or rejected against the
live evidence.

All six register rows are now filled and the workbook and PED copies agree cell
for cell.

Refs: #4
</commit_message>
<xml_diff>
--- a/docs/requirements/CivicConnect_M1_Registers.xlsx
+++ b/docs/requirements/CivicConnect_M1_Registers.xlsx
@@ -88,7 +88,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1753" uniqueCount="1013">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1753" uniqueCount="1021">
   <si>
     <t xml:space="preserve">CivicConnect - Milestone 1 controlled registers</t>
   </si>
@@ -3127,6 +3127,30 @@
   </si>
   <si>
     <t xml:space="preserve">The first attempt was rejected because it was not vector source that could be regenerated: the initial figure was a canvas rendering rather than SVG. It was redone as SVG generated from a Python script and rendered to PNG, so a marker can be moved by editing the source and re-rendering rather than by redrawing the image. Two discrepancies were then found on checking and are recorded rather than silently corrected. (1) Figure 1 names one gated decision per concern, but the Decision Log records FEC-01 and FEC-06 as gating DEC-009 as well as DEC-011, since DEC-009 requires the record-level authorisation shape from FEC-01 and the reporting load position from FEC-06; the figure understates those two rows by one decision. The Forward Considerations sheet also cites DEC-010 in the Links column for FEC-03 and FEC-05 but cites no decision for FEC-01 or FEC-06, so that link is recorded in the Decision Log only. (2) In Figure 2 the single New to In Progress arc carries two stacked labels while the Assigned self-loop carries none, so 'reassign to a different staff member' reads as belonging to the wrong transition; recorded as issue #27 and carried as a known limitation in s16.1 rather than corrected, since the diagram source is not held in the repository. All twelve transitions, their directions, authorised roles and guard conditions are otherwise correct.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">2026-09-09</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Tristan Roets</t>
+  </si>
+  <si>
+    <t xml:space="preserve">ChatGPT (OpenAI, GPT-5.6 Sol)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Reviewing M1 GitHub pull requests and preparing Risk Register and Forward Engineering Consideration evidence</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Assisted with identifying review blockers, checking traceability and governance issues, drafting review wording, and structuring Risk Register and FEC notes.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Compared the recommendations against the live GitHub pull requests, current main branch, CONTRIBUTING.md, issue requirements, and the controlled workbook and PED before accepting or revising them.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Accepted after revision</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Some suggestions were based on incomplete or outdated repository state. These were rechecked against the live repository, corrected where necessary, and unsupported claims were rejected.</t>
   </si>
 </sst>
 </file>
@@ -4552,29 +4576,29 @@
       </c>
     </row>
     <row r="4" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A4" s="12" t="s">
-        <v>756</v>
-      </c>
-      <c r="B4" s="12" t="s">
-        <v>483</v>
-      </c>
-      <c r="C4" s="12" t="s">
-        <v>757</v>
-      </c>
-      <c r="D4" s="10" t="s">
-        <v>763</v>
-      </c>
-      <c r="E4" s="10" t="s">
-        <v>764</v>
-      </c>
-      <c r="F4" s="10" t="s">
-        <v>765</v>
-      </c>
-      <c r="G4" s="10" t="s">
-        <v>766</v>
-      </c>
-      <c r="H4" s="12" t="s">
-        <v>767</v>
+      <c r="A4" s="9" t="s">
+        <v>1013</v>
+      </c>
+      <c r="B4" s="9" t="s">
+        <v>1014</v>
+      </c>
+      <c r="C4" s="9" t="s">
+        <v>1015</v>
+      </c>
+      <c r="D4" s="9" t="s">
+        <v>1016</v>
+      </c>
+      <c r="E4" s="9" t="s">
+        <v>1017</v>
+      </c>
+      <c r="F4" s="9" t="s">
+        <v>1018</v>
+      </c>
+      <c r="G4" s="9" t="s">
+        <v>1019</v>
+      </c>
+      <c r="H4" s="9" t="s">
+        <v>1020</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">

</xml_diff>

<commit_message>
docs: name the three approvers on the baseline sign-off
The three approval rows read "Team approval - [Member 1]" and so on, in the
workbook sheet and the PED s16 mirror. The names were never unknown; only the
approvals are outstanding.

They now carry the registered members. The Signature and date column stays
empty, as do the date, the six readiness fields, the outcome, the conditions
and the assessor decision, because the gate is on 10 September and none of
those has happened.

The distinction matters for how the sheet reads. Placeholders where the names
belong make a sign-off look unfinished; named approvers with empty signature
fields make it look like what it is, a gate that has not yet been held. Master
Brief s23 values honest incompleteness over the appearance of completeness, but
that only holds when the incompleteness is the real kind.

Refs: #7, Master Brief Appendix D
</commit_message>
<xml_diff>
--- a/docs/requirements/CivicConnect_M1_Registers.xlsx
+++ b/docs/requirements/CivicConnect_M1_Registers.xlsx
@@ -88,7 +88,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1753" uniqueCount="1013">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1753" uniqueCount="1016">
   <si>
     <t xml:space="preserve">CivicConnect - Milestone 1 controlled registers</t>
   </si>
@@ -3127,6 +3127,15 @@
   </si>
   <si>
     <t xml:space="preserve">The first attempt was rejected because it was not vector source that could be regenerated: the initial figure was a canvas rendering rather than SVG. It was redone as SVG generated from a Python script and rendered to PNG, so a marker can be moved by editing the source and re-rendering rather than by redrawing the image. Two discrepancies were then found on checking and are recorded rather than silently corrected. (1) Figure 1 names one gated decision per concern, but the Decision Log records FEC-01 and FEC-06 as gating DEC-009 as well as DEC-011, since DEC-009 requires the record-level authorisation shape from FEC-01 and the reporting load position from FEC-06; the figure understates those two rows by one decision. The Forward Considerations sheet also cites DEC-010 in the Links column for FEC-03 and FEC-05 but cites no decision for FEC-01 or FEC-06, so that link is recorded in the Decision Log only. (2) In Figure 2 the single New to In Progress arc carries two stacked labels while the Assigned self-loop carries none, so 'reassign to a different staff member' reads as belonging to the wrong transition; recorded as issue #27 and carried as a known limitation in s16.1 rather than corrected, since the diagram source is not held in the repository. All twelve transitions, their directions, authorised roles and guard conditions are otherwise correct.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Team approval - Jean Smit</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Team approval - Tristan Roets</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Team approval - Darius Mushi</t>
   </si>
 </sst>
 </file>
@@ -5828,7 +5837,7 @@
     </row>
     <row r="16" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A16" s="10" t="s">
-        <v>934</v>
+        <v>1013</v>
       </c>
       <c r="B16" s="10" t="s">
         <v>935</v>
@@ -5836,7 +5845,7 @@
     </row>
     <row r="17" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A17" s="9" t="s">
-        <v>936</v>
+        <v>1014</v>
       </c>
       <c r="B17" s="9" t="s">
         <v>935</v>
@@ -5844,7 +5853,7 @@
     </row>
     <row r="18" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A18" s="10" t="s">
-        <v>937</v>
+        <v>1015</v>
       </c>
       <c r="B18" s="10" t="s">
         <v>935</v>

</xml_diff>

<commit_message>
docs: complete Tristan AI Usage Register entry (#39)
Records Tristan Roets's M1 AI-assisted work in the controlled register and the
PED s14.2 mirror: the engineering task, what the assistant contributed, the
independent verification applied, and what was accepted after revision or
rejected.

Content supplied by Tristan Roets. Committed from Jean Smit's account because
he could not reach a machine tonight, and at his explicit request the commit is
not attributed to him: the authorship reflects who made the commit, and this
message records whose work it is.

His verification is checked against the live repository rather than asserted,
and the issues-found column records that some assistant output rested on an
outdated view of repository state and was corrected or rejected against the
live evidence.

All six register rows are now filled and the workbook and PED copies agree cell
for cell.

Refs: #4
</commit_message>
<xml_diff>
--- a/docs/requirements/CivicConnect_M1_Registers.xlsx
+++ b/docs/requirements/CivicConnect_M1_Registers.xlsx
@@ -88,7 +88,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1753" uniqueCount="1013">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1753" uniqueCount="1021">
   <si>
     <t xml:space="preserve">CivicConnect - Milestone 1 controlled registers</t>
   </si>
@@ -3127,6 +3127,30 @@
   </si>
   <si>
     <t xml:space="preserve">The first attempt was rejected because it was not vector source that could be regenerated: the initial figure was a canvas rendering rather than SVG. It was redone as SVG generated from a Python script and rendered to PNG, so a marker can be moved by editing the source and re-rendering rather than by redrawing the image. Two discrepancies were then found on checking and are recorded rather than silently corrected. (1) Figure 1 names one gated decision per concern, but the Decision Log records FEC-01 and FEC-06 as gating DEC-009 as well as DEC-011, since DEC-009 requires the record-level authorisation shape from FEC-01 and the reporting load position from FEC-06; the figure understates those two rows by one decision. The Forward Considerations sheet also cites DEC-010 in the Links column for FEC-03 and FEC-05 but cites no decision for FEC-01 or FEC-06, so that link is recorded in the Decision Log only. (2) In Figure 2 the single New to In Progress arc carries two stacked labels while the Assigned self-loop carries none, so 'reassign to a different staff member' reads as belonging to the wrong transition; recorded as issue #27 and carried as a known limitation in s16.1 rather than corrected, since the diagram source is not held in the repository. All twelve transitions, their directions, authorised roles and guard conditions are otherwise correct.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">2026-09-09</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Tristan Roets</t>
+  </si>
+  <si>
+    <t xml:space="preserve">ChatGPT (OpenAI, GPT-5.6 Sol)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Reviewing M1 GitHub pull requests and preparing Risk Register and Forward Engineering Consideration evidence</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Assisted with identifying review blockers, checking traceability and governance issues, drafting review wording, and structuring Risk Register and FEC notes.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Compared the recommendations against the live GitHub pull requests, current main branch, CONTRIBUTING.md, issue requirements, and the controlled workbook and PED before accepting or revising them.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Accepted after revision</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Some suggestions were based on incomplete or outdated repository state. These were rechecked against the live repository, corrected where necessary, and unsupported claims were rejected.</t>
   </si>
 </sst>
 </file>
@@ -4552,29 +4576,29 @@
       </c>
     </row>
     <row r="4" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A4" s="12" t="s">
-        <v>756</v>
-      </c>
-      <c r="B4" s="12" t="s">
-        <v>483</v>
-      </c>
-      <c r="C4" s="12" t="s">
-        <v>757</v>
-      </c>
-      <c r="D4" s="10" t="s">
-        <v>763</v>
-      </c>
-      <c r="E4" s="10" t="s">
-        <v>764</v>
-      </c>
-      <c r="F4" s="10" t="s">
-        <v>765</v>
-      </c>
-      <c r="G4" s="10" t="s">
-        <v>766</v>
-      </c>
-      <c r="H4" s="12" t="s">
-        <v>767</v>
+      <c r="A4" s="9" t="s">
+        <v>1013</v>
+      </c>
+      <c r="B4" s="9" t="s">
+        <v>1014</v>
+      </c>
+      <c r="C4" s="9" t="s">
+        <v>1015</v>
+      </c>
+      <c r="D4" s="9" t="s">
+        <v>1016</v>
+      </c>
+      <c r="E4" s="9" t="s">
+        <v>1017</v>
+      </c>
+      <c r="F4" s="9" t="s">
+        <v>1018</v>
+      </c>
+      <c r="G4" s="9" t="s">
+        <v>1019</v>
+      </c>
+      <c r="H4" s="9" t="s">
+        <v>1020</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">

</xml_diff>